<commit_message>
Cadre la feature F01, socle plateforme
Fiche à l'état « à cadrer » : neuf identifiants du backlog, 38 règles
métier sourcées, 39 critères d'acceptation en cas concrets, hors
périmètre, dépendances, dix questions à trancher.

F01 passe à « Cadrage » dans le suivi.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ViEcD75tDcp4v6Y1YDjAs8
</commit_message>
<xml_diff>
--- a/docs/suivi-features.xlsx
+++ b/docs/suivi-features.xlsx
@@ -39,9 +39,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="165" formatCode="0 %"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="166" formatCode="0 %"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -153,10 +154,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -167,7 +168,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2925,11 +2926,13 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Waiting</t>
+          <t>Cadrage</t>
         </is>
       </c>
       <c r="G2" s="4" t="n"/>
-      <c r="H2" s="17" t="n"/>
+      <c r="H2" s="17" t="n">
+        <v>46285</v>
+      </c>
       <c r="I2" s="17" t="n"/>
       <c r="J2" s="17" t="n"/>
       <c r="K2" s="17" t="n"/>
@@ -2944,7 +2947,11 @@
         <f>IF(AND(M2&lt;&gt;"",O2&lt;&gt;""),O2-M2,"")</f>
         <v/>
       </c>
-      <c r="Q2" s="4" t="n"/>
+      <c r="Q2" s="4" t="inlineStr">
+        <is>
+          <t>Fiche rédigée, 10 questions en attente</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">

</xml_diff>

<commit_message>
F01 : étape 2 close, rôle Administrateur et granularité des permissions
Benchmark tranché : sept écarts intégrés dans les règles (auteur système
et parent dans l'audit, journal jamais purgé, recherche dans le journal,
appareil de confiance, codes de secours, fermeture des sessions,
permission d'export distincte), trois écartés.

B8 passe du backlog à F01 : un sixième rôle, Administrateur, titulaire du
compte, octroie et retire les droits utilisateur par utilisateur, le rôle
restant le jeu par défaut. Granularité fixée : un droit par décision
sensible et par écran, jamais par champ ; grammaire domaine.objet.action,
droits paramétrés pour les plafonds. Décision 0028 ; glossaire, gabarit,
processus et backend/CLAUDE.md complétés.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ViEcD75tDcp4v6Y1YDjAs8
</commit_message>
<xml_diff>
--- a/docs/suivi-features.xlsx
+++ b/docs/suivi-features.xlsx
@@ -2933,7 +2933,9 @@
       <c r="H2" s="17" t="n">
         <v>46285</v>
       </c>
-      <c r="I2" s="17" t="n"/>
+      <c r="I2" s="17" t="n">
+        <v>46285</v>
+      </c>
       <c r="J2" s="17" t="n"/>
       <c r="K2" s="17" t="n"/>
       <c r="L2" s="17" t="n"/>
@@ -2949,7 +2951,7 @@
       </c>
       <c r="Q2" s="4" t="inlineStr">
         <is>
-          <t>Fiche rédigée, 10 questions en attente</t>
+          <t>Étapes 1 et 2 closes ; étape 3 (plan) à faire</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
F01 : plan validé, choix structurants du socle actés
Les huit points majeurs sont validés (décision 0029), sauf le client S3,
non retenu tant que l'hébergeur n'est pas choisi : F01 livre l'interface
de stockage avec disque et mémoire. Dépendances validées : Bouncy Castle,
fastexcel, angularx-qrcode. Les CLAUDE.md backend et frontend intègrent
l'audit bloquant, le compte utilisateur global et les dépendances.

F01 passe à « Dev » dans le suivi.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ViEcD75tDcp4v6Y1YDjAs8
</commit_message>
<xml_diff>
--- a/docs/suivi-features.xlsx
+++ b/docs/suivi-features.xlsx
@@ -2926,7 +2926,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Cadrage</t>
+          <t>Dev</t>
         </is>
       </c>
       <c r="G2" s="4" t="n"/>
@@ -2936,7 +2936,9 @@
       <c r="I2" s="17" t="n">
         <v>46285</v>
       </c>
-      <c r="J2" s="17" t="n"/>
+      <c r="J2" s="17" t="n">
+        <v>46285</v>
+      </c>
       <c r="K2" s="17" t="n"/>
       <c r="L2" s="17" t="n"/>
       <c r="M2" s="17" t="n"/>
@@ -2951,7 +2953,7 @@
       </c>
       <c r="Q2" s="4" t="inlineStr">
         <is>
-          <t>Étapes 1 et 2 closes ; étape 3 (plan) à faire</t>
+          <t>Plan validé ; étape 4 (tests d'abord) à faire</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
F01 : livraison — modèle de données, décision 0030, fiche et suivi
- docs/modele-donnees.md : les quatorze tables du socle, avec leurs attributs
  arrêtés et les deux enseignements qui valent pour le modèle à venir ;
- décision 0030 : les six points tranchés pendant l'implémentation ;
- fiche F01 : bilan de l'étape 5, les trois défauts trouvés à l'usage et le test
  qui ferme chacun, ce qui reste à faire ;
- suivi : F01 passée à « In test », en attente de validation.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ViEcD75tDcp4v6Y1YDjAs8
</commit_message>
<xml_diff>
--- a/docs/suivi-features.xlsx
+++ b/docs/suivi-features.xlsx
@@ -39,10 +39,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0 %"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="166" formatCode="0 %"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -144,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -154,10 +153,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -169,6 +168,8 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -699,7 +700,7 @@
         <f>COUNTIFS(Features!$C$2:$C$74,$A6,Features!$F$2:$F$74,"Production")</f>
         <v/>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="18">
         <f>IF($D6=0,"",$I6/$D6)</f>
         <v/>
       </c>
@@ -747,7 +748,7 @@
         <f>COUNTIFS(Features!$C$2:$C$74,$A7,Features!$F$2:$F$74,"Production")</f>
         <v/>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="18">
         <f>IF($D7=0,"",$I7/$D7)</f>
         <v/>
       </c>
@@ -795,7 +796,7 @@
         <f>COUNTIFS(Features!$C$2:$C$74,$A8,Features!$F$2:$F$74,"Production")</f>
         <v/>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="18">
         <f>IF($D8=0,"",$I8/$D8)</f>
         <v/>
       </c>
@@ -843,7 +844,7 @@
         <f>COUNTIFS(Features!$C$2:$C$74,$A9,Features!$F$2:$F$74,"Production")</f>
         <v/>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="18">
         <f>IF($D9=0,"",$I9/$D9)</f>
         <v/>
       </c>
@@ -891,7 +892,7 @@
         <f>COUNTIFS(Features!$C$2:$C$74,$A10,Features!$F$2:$F$74,"Production")</f>
         <v/>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="18">
         <f>IF($D10=0,"",$I10/$D10)</f>
         <v/>
       </c>
@@ -939,7 +940,7 @@
         <f>COUNTIFS(Features!$C$2:$C$74,$A11,Features!$F$2:$F$74,"Production")</f>
         <v/>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="18">
         <f>IF($D11=0,"",$I11/$D11)</f>
         <v/>
       </c>
@@ -987,7 +988,7 @@
         <f>COUNTIFS(Features!$C$2:$C$74,$A12,Features!$F$2:$F$74,"Production")</f>
         <v/>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="18">
         <f>IF($D12=0,"",$I12/$D12)</f>
         <v/>
       </c>
@@ -1035,7 +1036,7 @@
         <f>COUNTIFS(Features!$C$2:$C$74,$A13,Features!$F$2:$F$74,"Production")</f>
         <v/>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="18">
         <f>IF($D13=0,"",$I13/$D13)</f>
         <v/>
       </c>
@@ -1083,7 +1084,7 @@
         <f>COUNTIFS(Features!$C$2:$C$74,$A14,Features!$F$2:$F$74,"Production")</f>
         <v/>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="18">
         <f>IF($D14=0,"",$I14/$D14)</f>
         <v/>
       </c>
@@ -1123,7 +1124,7 @@
         <f>SUM(I6:I14)</f>
         <v/>
       </c>
-      <c r="J15" s="8">
+      <c r="J15" s="19">
         <f>IF($D15=0,"",$I15/$D15)</f>
         <v/>
       </c>
@@ -2926,21 +2927,39 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Dev</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="17" t="n">
-        <v>46285</v>
-      </c>
-      <c r="I2" s="17" t="n">
-        <v>46285</v>
-      </c>
-      <c r="J2" s="17" t="n">
-        <v>46285</v>
-      </c>
-      <c r="K2" s="17" t="n"/>
-      <c r="L2" s="17" t="n"/>
+          <t>In test</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="H2" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="I2" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="J2" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="K2" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="L2" s="17" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
       <c r="M2" s="17" t="n"/>
       <c r="N2" s="4">
         <f>IF(AND(H2&lt;&gt;"",M2&lt;&gt;""),M2-H2,"")</f>

</xml_diff>